<commit_message>
Thêm ảnh chụp giá trị vào tab 0_README
File do openpyxl sinh ra không mang giá trị cache, nên trình xem nhẹ có thể
hiện ô trống dù Excel, LibreOffice và Google Sheets đều tính lại khi mở.
Bảng ảnh chụp giữ đủ 5 con số bắt buộc kèm địa chỉ ô gốc để truy ngược.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2A202601821_LeQuangHuy_Day25_model.xlsx
+++ b/2A202601821_LeQuangHuy_Day25_model.xlsx
@@ -612,8 +612,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -923,11 +923,366 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>ẢNH CHỤP GIÁ TRỊ TẠI NGÀY LẬP — 27/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Công thức SỐNG nằm ở các tab 1–4; đây chỉ là ảnh chụp để đọc được cả khi mở bằng trình xem không tính công thức. Nếu sửa ô vàng, hãy đọc số ở tab tương ứng chứ không đọc bảng này.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Cost/Job</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="inlineStr">
+        <is>
+          <t>0,0627 $ = 1.629 ₫</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>1_Cost_Job!B98</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>chia cho 95.284 job HOÀN THÀNH</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nếu chia nhầm cho 140.000 ca đã thử</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>0,0427 $</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>1_Cost_Job!B100</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>rẻ giả 31,9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Tổng COGS / tháng</t>
+        </is>
+      </c>
+      <c r="B31" s="31" t="inlineStr">
+        <is>
+          <t>5.971,53 $ = 155,3tr ₫</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>1_Cost_Job!B96</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>LLM 32,6% · Retry 2,3% · Infra 8,2% · HITL QA 45,1% · Khác 11,7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Giá sàn = 3 × Cost/Job</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>0,1880 $ = 4.888 ₫</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>2_Pricing!B17</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Giá bán bình quân / job</t>
+        </is>
+      </c>
+      <c r="B33" s="31" t="inlineStr">
+        <is>
+          <t>0,2309 $ = 6.004 ₫</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>2_Pricing!B12</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>NẰM TRONG VÙNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Giá trần = 25% giá trị tạo ra</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>0,3278 $ = 8.523 ₫</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>2_Pricing!B24</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Doanh thu / ví / tháng</t>
+        </is>
+      </c>
+      <c r="B35" s="31" t="inlineStr">
+        <is>
+          <t>22.002,46 $ = 572,1tr ₫</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>2_Pricing!B10</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>ta thu 17,6% giá trị · ROI khách 5,7x</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Gross Margin</t>
+        </is>
+      </c>
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>72,86%</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>2_Pricing!B33</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>ĐẠT ngưỡng 60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Giá bán / Cost/Job</t>
+        </is>
+      </c>
+      <c r="B37" s="31" t="inlineStr">
+        <is>
+          <t>3,68x</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>2_Pricing!B34</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>ĐẠT ngưỡng 3,00x</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Breakeven — hồ sơ duyệt-lần-đầu (3x)</t>
+        </is>
+      </c>
+      <c r="B38" s="31" t="inlineStr">
+        <is>
+          <t>46,67%</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>2_Pricing!B43</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>ĐO THẬT 27/08/2026 = 1,03% → CHƯA ĐẠT</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Breakeven — hồ sơ duyệt-lần-đầu (GM 60%)</t>
+        </is>
+      </c>
+      <c r="B39" s="31" t="inlineStr">
+        <is>
+          <t>28,89%</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>2_Pricing!B44</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Gross Margin ở Biến thể B</t>
+        </is>
+      </c>
+      <c r="B40" s="31" t="inlineStr">
+        <is>
+          <t>−61,27%</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>2_Pricing!B55</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>cần tỷ lệ hoàn thành 94,1% mới về 60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Điểm Attribution / Autonomy</t>
+        </is>
+      </c>
+      <c r="B41" s="31" t="inlineStr">
+        <is>
+          <t>2/5 và 1/5</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>3_Value_Metric!B9,B18</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>ma trận trỏ SEAT/HYBRID</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ngân sách CAC</t>
+        </is>
+      </c>
+      <c r="B42" s="31" t="inlineStr">
+        <is>
+          <t>384.742 $</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>4_Channel_Fit!B8</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>CAC thực tế 44.800 $ → dư 8,59x</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CAC payback · LTV/CAC</t>
+        </is>
+      </c>
+      <c r="B43" s="31" t="inlineStr">
+        <is>
+          <t>2,79 tháng · 17,9x</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>4_Channel_Fit!B28,B31</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>ĐẠT cả hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Deal / AE / ngày làm việc</t>
+        </is>
+      </c>
+      <c r="B44" s="31" t="inlineStr">
+        <is>
+          <t>0,0012</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>4_Channel_Fit!B18</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>Sales-Led khả thi về số học</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A24:D24"/>
     <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A24:D24"/>
     <mergeCell ref="A10:D10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -941,7 +1296,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F110"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -2465,7 +2820,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H80"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -3736,7 +4091,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F44"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -4267,7 +4622,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F50"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -4995,7 +5350,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -5370,7 +5725,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E49"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Sửa hai ô ghi chú bắt đầu bằng dấu = khiến Excel hiện #NAME?
Ô 1_Cost_Job!D98 và 6_Benchmarks!C10 chứa văn bản mở đầu bằng '=' nên
openpyxl ghi chúng vào phần tử <f>, Excel sẽ cố phân tích như công thức.

Kèm theo: đã dựng bộ tính riêng đánh giá toàn bộ 168 ô công thức trong
workbook và đối chiếu 31 chỉ số chính với mô hình Python — khớp tuyệt đối,
không còn ô nào lỗi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2A202601821_LeQuangHuy_Day25_model.xlsx
+++ b/2A202601821_LeQuangHuy_Day25_model.xlsx
@@ -2617,9 +2617,10 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="D98" s="11">
-        <f> tổng COGS chia cho ô 'Số job hoàn thành' ở S2</f>
-        <v/>
+      <c r="D98" s="11" t="inlineStr">
+        <is>
+          <t>Lấy tổng COGS chia cho ô 'Số job hoàn thành' ở S2</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -5875,9 +5876,10 @@
           <t>01:00–04:00 và 06:00–10:00 UTC, thứ Hai–thứ Sáu</t>
         </is>
       </c>
-      <c r="C10" s="44">
-        <f> 08–11h và 13–17h giờ VN</f>
-        <v/>
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>tức 08–11h và 13–17h giờ VN</t>
+        </is>
       </c>
       <c r="D10" s="44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Xác minh benchmark Zendesk tại nguồn, thay trích dẫn gián tiếp
Trang tài liệu Zendesk (kiểm tra 27/08/2026) cho ba bậc automated resolution:
assisted escalation và contained resolution KHÔNG trừ hạn mức, chỉ verified
resolution mới trừ và phải qua LLM kiểm chứng. Cửa sổ kết thúc hội thoại:
72h email, 2h messaging (chỉnh được tới 72h), ngay khi cúp máy với thoại.
Trang này không công bố đơn giá — con số 1,50 $/resolution lưu hành là từ
blog, nên bỏ khỏi bài.

Ba bậc đó gần trùng ba lớp ca của WalletCare, nên thêm một đoạn đối chiếu ở
3_Value_Metric: Zendesk cũng kết luận ca có người can thiệp không được tính
tiền như ca AI tự đóng.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2A202601821_LeQuangHuy_Day25_model.xlsx
+++ b/2A202601821_LeQuangHuy_Day25_model.xlsx
@@ -4091,7 +4091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -4513,12 +4513,12 @@
       </c>
       <c r="C39" s="39" t="inlineStr">
         <is>
-          <t>3 bậc automated resolution; định nghĩa gắn với cửa sổ khách không mở lại: 72 giờ email · 2 giờ messaging · ngay lập tức với thoại.</t>
+          <t>Ba bậc, chỉ MỘT bậc bị trừ vào hạn mức: assisted escalation (người hoàn tất — không trừ) · contained resolution (AI xử lý xong, khách không hỏi thêm — không trừ) · verified resolution (AI giải quyết xong, có LLM kiểm chứng — TRỪ hạn mức). Cửa sổ kết thúc hội thoại: 72 giờ email · 2 giờ messaging (chỉnh được tới 72 giờ) · ngay khi cúp máy với thoại. Trang này KHÔNG công bố đơn giá.</t>
         </is>
       </c>
       <c r="D39" s="40" t="inlineStr">
         <is>
-          <t>https://www.zendesk.com/blog/ai/agentic-ai/outcome-based-pricing/</t>
+          <t>https://support.zendesk.com/hc/en-us/articles/9570369117338-About-automated-resolution-tiers</t>
         </is>
       </c>
     </row>
@@ -4590,14 +4590,27 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>Ba bậc của Zendesk gần như trùng ba lớp ca của ta</t>
+        </is>
+      </c>
+      <c r="B45" s="39" t="inlineStr">
+        <is>
+          <t>Kiểm tra trang tài liệu Zendesk ngày 27/08/2026: assisted escalation (người hoàn tất) không bị trừ hạn mức · contained resolution (AI xử lý xong, khách không hỏi thêm) không bị trừ · verified resolution mới bị trừ. Tức Zendesk cũng kết luận rằng ca có người can thiệp KHÔNG được tính tiền như ca AI tự đóng. Ta đi xa hơn một bước và tính tiền cho đường hồ sơ, nhưng chỉ khi nó được duyệt ngay lần trình đầu — vì với FIN-05, hồ sơ điều tra chính là sản phẩm ví bỏ tiền mua, không phải phần thừa của một ca thất bại.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="B31:D31"/>
     <mergeCell ref="A36:F36"/>
+    <mergeCell ref="B45:D45"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A12:F12"/>
@@ -6120,7 +6133,7 @@
       </c>
       <c r="B23" s="42" t="inlineStr">
         <is>
-          <t>3 bậc automated resolution; định nghĩa gắn cửa sổ mở lại 72h/2h/ngay</t>
+          <t>Ba bậc: assisted escalation · contained resolution · verified resolution — chỉ bậc thứ ba bị trừ hạn mức và phải qua LLM kiểm chứng. Cửa sổ kết thúc: 72h email · 2h messaging (chỉnh tới 72h) · ngay khi cúp máy. KHÔNG công bố đơn giá trên trang này; con số 1,50 $/resolution lưu hành là từ blog, không phải trang giá.</t>
         </is>
       </c>
       <c r="C23" s="44" t="inlineStr">
@@ -6130,12 +6143,12 @@
       </c>
       <c r="D23" s="44" t="inlineStr">
         <is>
-          <t>26/08/2026 (theo §3.5 Lab)</t>
+          <t>27/08/2026</t>
         </is>
       </c>
       <c r="E23" s="45" t="inlineStr">
         <is>
-          <t>https://www.zendesk.com/blog/ai/agentic-ai/outcome-based-pricing/</t>
+          <t>https://support.zendesk.com/hc/en-us/articles/9570369117338-About-automated-resolution-tiers</t>
         </is>
       </c>
     </row>

</xml_diff>